<commit_message>
feat: add ExcelSpreadsheetView UI with formula bar and bottom sheet tabs; add Sheet Khoan 4.5 TT20
</commit_message>
<xml_diff>
--- a/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_CHUAN_F1_100PCT.xlsx
+++ b/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_CHUAN_F1_100PCT.xlsx
@@ -16,8 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhân công" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Công cụ dụng cụ" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Máy thi công" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="THDT hạng mục" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đơn giá chi tiết" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khoản 4.5 TT20" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="THDT hạng mục" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đơn giá chi tiết" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -180,19 +181,19 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -804,7 +805,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>2.1.2 DỰ KIẾN KHỐI LƯỢNG NỘI DUNG CÔNG VIỆC PHỤC VỤ LẤY MẪU TẠI HIỆN TRƯỜNG (KHOẢN 4.5 TT20)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="n"/>
+      <c r="C1" s="6" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="6" t="n"/>
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="6" t="n"/>
+      <c r="I1" s="6" t="n"/>
+      <c r="J1" s="6" t="n"/>
+      <c r="K1" s="6" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>(Căn cứ theo Mục 2.1.2 Báo cáo PAKT gửi ngày 28/10/2026 của KTAT NMNĐ Vĩnh Tân 4 và Khoản 4.5 TT 20/2017)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7">
+        <f>'Công trình'!A3</f>
+        <v/>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <f>'Công trình'!A4</f>
+        <v/>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Nội dung công việc / Chức danh / Phương tiện</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Đơn vị</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 1</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 2</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 3</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 4</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Tổng cộng</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Đơn giá (VNĐ)</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Thành tiền (VNĐ)</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Ghi chú nghiệp vụ KTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>ĐỐI VỚI QUAN TRẮC MÔI TRƯỜNG ĐỊNH KỲ THEO GIẤY PHÉP MÔI TRƯỜNG</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr"/>
+      <c r="D7" s="28" t="inlineStr"/>
+      <c r="E7" s="28" t="inlineStr"/>
+      <c r="F7" s="28" t="inlineStr"/>
+      <c r="G7" s="28" t="inlineStr"/>
+      <c r="H7" s="28" t="inlineStr"/>
+      <c r="I7" s="18" t="inlineStr"/>
+      <c r="J7" s="18" t="inlineStr"/>
+      <c r="K7" s="22" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Nhân sự thực hiện hiện trường</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Người</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="H8" s="20">
+        <f>SUM(D8:G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="11" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>QTV hạng IV không quá 30% đội ngũ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Số chuyến xe phương tiện di chuyển</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Chuyến</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="20">
+        <f>SUM(D9:G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="J9" s="11">
+        <f>ROUND(H9*I9, 0)</f>
+        <v/>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>Bảo quản hỏa tốc Coliform, BOD5, CrVI (24h-48h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Số ngày đi/về của mỗi đợt</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="20">
+        <f>SUM(D10:G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>Hà Nội - Bình Thuận khứ hồi (2.800 km)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Số công di chuyển (Số người × Số ngày đi/về)</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Công</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="H11" s="20">
+        <f>SUM(D11:G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>319090</v>
+      </c>
+      <c r="J11" s="11">
+        <f>ROUND(H11*I11, 0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>Tính lương theo chuẩn 22 ngày QĐ 80/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>VII</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Khối lượng lưu trú tại hiện trường</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Đêm</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" s="20">
+        <f>SUM(D12:G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>450000</v>
+      </c>
+      <c r="J12" s="11">
+        <f>ROUND(H12*I12, 0)</f>
+        <v/>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>Nhóm KKXQ 5 người x 5 ngày (TT 40/2017/TT-BTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>VIII</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Khối lượng văn phòng phẩm, in ấn kết quả</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>đồng</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H13" s="20">
+        <f>SUM(D13:G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="11">
+        <f>ROUND(H13*I13, 0)</f>
+        <v/>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>Trọn gói in ấn kết quả phân tích từng đợt</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>CHƯƠNG TRÌNH QUAN TRẮC MÔI TRƯỜNG ĐỐI CHỨNG</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr"/>
+      <c r="D14" s="28" t="inlineStr"/>
+      <c r="E14" s="28" t="inlineStr"/>
+      <c r="F14" s="28" t="inlineStr"/>
+      <c r="G14" s="28" t="inlineStr"/>
+      <c r="H14" s="28" t="inlineStr"/>
+      <c r="I14" s="18" t="inlineStr"/>
+      <c r="J14" s="18" t="inlineStr"/>
+      <c r="K14" s="22" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Nhân sự thực hiện hiện trường</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Người</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="20">
+        <f>SUM(D15:G15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="11" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr">
+        <is>
+          <t>QTV hạng IV không quá 30% đội ngũ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Số chuyến xe phương tiện di chuyển</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Chuyến</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="20">
+        <f>SUM(D16:G16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="J16" s="11">
+        <f>ROUND(H16*I16, 0)</f>
+        <v/>
+      </c>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>Vận chuyển mẫu nước thải, khí thải, nước biển</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Số ngày đi/về của mỗi đợt</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" s="20">
+        <f>SUM(D17:G17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="11" t="inlineStr"/>
+      <c r="J17" s="11" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>Hà Nội - Bình Thuận khứ hồi (2.800 km)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Số công di chuyển (Số người × Số ngày đi/về)</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Công</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="G18" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="H18" s="20">
+        <f>SUM(D18:G18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>319090</v>
+      </c>
+      <c r="J18" s="11">
+        <f>ROUND(H18*I18, 0)</f>
+        <v/>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>Đợt 1: 15 người x 4 ngày; Đợt 2: 12 người x 4 ngày...</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>VII</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Khối lượng lưu trú tại hiện trường</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Đêm</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="H19" s="20">
+        <f>SUM(D19:G19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>450000</v>
+      </c>
+      <c r="J19" s="11">
+        <f>ROUND(H19*I19, 0)</f>
+        <v/>
+      </c>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>Lưu trú Tuy Phong theo Thông tư 40/2017/TT-BTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>VIII</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Khối lượng văn phòng phẩm, in ấn kết quả</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>đồng</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G20" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H20" s="20">
+        <f>SUM(D20:G20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="11">
+        <f>ROUND(H20*I20, 0)</f>
+        <v/>
+      </c>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>Trọn gói in ấn kết quả phân tích đối chứng</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>CHI PHÍ KỸ THUẬT NGOÀI ĐỊNH MỨC KHÁC THEO KHOẢN 4.5 TT20</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr"/>
+      <c r="D21" s="28" t="inlineStr"/>
+      <c r="E21" s="28" t="inlineStr"/>
+      <c r="F21" s="28" t="inlineStr"/>
+      <c r="G21" s="28" t="inlineStr"/>
+      <c r="H21" s="28" t="inlineStr"/>
+      <c r="I21" s="18" t="inlineStr"/>
+      <c r="J21" s="18" t="inlineStr"/>
+      <c r="K21" s="22" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Sàn thao tác, giàn giáo, lỗ lấy mẫu khí thải ống khói lò hơi</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>trọn gói</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>280000000</v>
+      </c>
+      <c r="J22" s="11" t="n">
+        <v>280000000</v>
+      </c>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>Định mức Xây dựng TT 12/2021/TT-BXD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Thuê tàu biển chuyên dụng khảo sát nước biển xa bờ bãi xỉ</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>ngày tàu</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="J23" s="11">
+        <f>ROUND(H23*I23, 0)</f>
+        <v/>
+      </c>
+      <c r="K23" s="1" t="inlineStr">
+        <is>
+          <t>Tối thiểu 3 báo giá cạnh tranh NĐ 24/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr"/>
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>CỘNG CHI PHÍ TÍNH RIÊNG NGOÀI ĐỊNH MỨC (KHOẢN 4.5 TT20):</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="inlineStr"/>
+      <c r="D24" s="29" t="inlineStr"/>
+      <c r="E24" s="29" t="inlineStr"/>
+      <c r="F24" s="29" t="inlineStr"/>
+      <c r="G24" s="29" t="inlineStr"/>
+      <c r="H24" s="29" t="inlineStr"/>
+      <c r="I24" s="26" t="inlineStr"/>
+      <c r="J24" s="26">
+        <f>J9+J11+J12+J13+J16+J18+J19+J20+J22+J23</f>
+        <v/>
+      </c>
+      <c r="K24" s="25" t="inlineStr">
+        <is>
+          <t>Tổng chi phí tính riêng đưa vào THDT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -857,14 +1715,14 @@
       <c r="E4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="n"/>
-      <c r="B5" s="28" t="n"/>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" s="30" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
@@ -884,7 +1742,7 @@
           <t>GIÁ TRỊ (VNĐ)</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>KÝ HIỆU</t>
         </is>
@@ -898,15 +1756,15 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Chi phí trực tiếp (T = VL + DC + NC + M)</t>
+          <t>Chi phí trực tiếp (T = VL + DC + NC + M + C_TR)</t>
         </is>
       </c>
       <c r="C7" s="1">
-        <f>"VL + DC + NC + M"</f>
+        <f>"VL + DC + NC + M + C_TR"</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>ROUND(D8+D10+D12+D14, 0)</f>
+        <f>ROUND(D8+D10+D12+D14+D16, 0)</f>
         <v/>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1082,13 +1940,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr"/>
-      <c r="B15" s="31" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr"/>
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve"> - Đơn giá máy thi công</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>Theo bảng tổng hợp máy thi công</t>
         </is>
@@ -1097,7 +1955,7 @@
         <f>'Máy thi công'!$G$80</f>
         <v/>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>MHT</t>
         </is>
@@ -1106,213 +1964,217 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Chi phí gián tiếp</t>
+          <t>Chi phí tính riêng ngoài định mức (Khoản 4.5 TT20)</t>
         </is>
       </c>
       <c r="C16" s="1">
-        <f>"C + TT"</f>
+        <f>"C_TR"</f>
         <v/>
       </c>
       <c r="D16" s="11">
-        <f>D16+D17</f>
+        <f>'Khoản 4.5 TT20'!$J$24</f>
         <v/>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>C_TR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Chi phí gián tiếp</t>
+        </is>
+      </c>
+      <c r="C17" s="1">
+        <f>"C + TT"</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>GT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>Chi phí chung</t>
         </is>
       </c>
-      <c r="C17" s="1">
+      <c r="C18" s="32">
         <f>"T x 20%"</f>
         <v/>
       </c>
-      <c r="D17" s="11">
+      <c r="D18" s="9">
         <f>ROUND(D6*'Hệ số'!$C$4, 0)</f>
         <v/>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E18" s="31" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>Chi phí một số công việc không xác định từ thiết kế</t>
         </is>
       </c>
-      <c r="C18" s="31">
+      <c r="C19" s="22">
         <f>"T x 2,5%"</f>
         <v/>
       </c>
-      <c r="D18" s="9">
+      <c r="D19" s="18">
         <f>ROUND(D6*'Hệ số'!$C$9, 0)</f>
         <v/>
       </c>
-      <c r="E18" s="30" t="inlineStr">
+      <c r="E19" s="28" t="inlineStr">
         <is>
           <t>TT</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>III</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Thu nhập chịu thuế tính trước</t>
         </is>
       </c>
-      <c r="C19" s="22">
+      <c r="C20" s="1">
         <f>"(T + GT) x 5,5%"</f>
         <v/>
       </c>
-      <c r="D19" s="18">
+      <c r="D20" s="11">
         <f>ROUND((D6+D15)*'Hệ số'!$C$8, 0)</f>
         <v/>
       </c>
-      <c r="E19" s="29" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="20" t="inlineStr"/>
-      <c r="B20" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr"/>
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>Chi phí trước thuế</t>
         </is>
       </c>
-      <c r="C20" s="1">
+      <c r="C21" s="22">
         <f>"T + GT + TL"</f>
         <v/>
       </c>
-      <c r="D20" s="11">
+      <c r="D21" s="18">
         <f>ROUND(D6+D15+D18, 0)</f>
         <v/>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E21" s="28" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>IV</t>
         </is>
       </c>
-      <c r="B21" s="22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Thuế giá trị gia tăng</t>
         </is>
       </c>
-      <c r="C21" s="22">
+      <c r="C22" s="1">
         <f>"G x 8%"</f>
         <v/>
       </c>
-      <c r="D21" s="18">
+      <c r="D22" s="11">
         <f>ROUND(D19*'Hệ số'!$C$10, 0)</f>
         <v/>
       </c>
-      <c r="E21" s="29" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>GTGT</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr"/>
-      <c r="B22" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr"/>
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>CHI PHÍ SAU THUẾ</t>
         </is>
       </c>
-      <c r="C22" s="1">
+      <c r="C23" s="22">
         <f>"G + GTGT"</f>
         <v/>
       </c>
-      <c r="D22" s="11">
+      <c r="D23" s="18">
         <f>ROUND(D19+D20, 0)</f>
         <v/>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>Gxd</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="29" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>Chi phí nhà tạm để ở và điều hành</t>
         </is>
       </c>
-      <c r="C23" s="22">
+      <c r="C24" s="25">
         <f>"G x 1,1% x (1 + 8%)"</f>
         <v/>
       </c>
-      <c r="D23" s="18">
+      <c r="D24" s="26">
         <f>ROUND(D19*'Hệ số'!$C$6*(1+'Hệ số'!$C$10), 0)</f>
         <v/>
       </c>
-      <c r="E23" s="29" t="inlineStr">
+      <c r="E24" s="29" t="inlineStr">
         <is>
           <t>LT</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr"/>
-      <c r="B24" s="25" t="inlineStr">
-        <is>
-          <t>TỔNG CỘNG KINH PHÍ GÓI THẦU</t>
-        </is>
-      </c>
-      <c r="C24" s="25">
-        <f>"Gxd + LT"</f>
-        <v/>
-      </c>
-      <c r="D24" s="26">
-        <f>ROUND(D21+D22, 0)</f>
-        <v/>
-      </c>
-      <c r="E24" s="32" t="inlineStr">
-        <is>
-          <t>TTS</t>
         </is>
       </c>
     </row>
@@ -1320,18 +2182,39 @@
       <c r="A25" s="6" t="inlineStr"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>TỔNG CỘNG KINH PHÍ GÓI THẦU</t>
+        </is>
+      </c>
+      <c r="C25" s="6">
+        <f>"Gxd + LT"</f>
+        <v/>
+      </c>
+      <c r="D25" s="6">
+        <f>ROUND(D21+D22, 0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>TTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
           <t>LÀM TRÒN (ĐẾN HÀNG NGHÌN ĐỒNG)</t>
         </is>
       </c>
-      <c r="C25" s="6">
+      <c r="C26" s="6">
         <f>"ROUND(D23, -3)"</f>
         <v/>
       </c>
-      <c r="D25" s="6">
+      <c r="D26" s="6">
         <f>ROUND(D23, -3)</f>
         <v/>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>LTR</t>
         </is>
@@ -1342,7 +2225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>